<commit_message>
add chart & setup run game
</commit_message>
<xml_diff>
--- a/rollforever/Assets/Excels/MonsterConfig.xlsx
+++ b/rollforever/Assets/Excels/MonsterConfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Idle-rpg\rollforever\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E31A054-E1FD-4336-9B5C-575207CC3991}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4923BB72-D56F-4C41-9DCB-65C385B42B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>id</t>
   </si>
@@ -85,6 +85,18 @@
   </si>
   <si>
     <t>1000101_prefab</t>
+  </si>
+  <si>
+    <t>Monster 2</t>
+  </si>
+  <si>
+    <t>1000102_prefab</t>
+  </si>
+  <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>Tanker</t>
   </si>
 </sst>
 </file>
@@ -418,113 +430,116 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.81640625" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" customWidth="1"/>
-    <col min="3" max="3" width="17.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.36328125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.36328125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="11.81640625" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" customWidth="1"/>
+    <col min="4" max="4" width="17.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="16.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" ht="16.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="O1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="S1" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1000101</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>18</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>19</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>10101</v>
       </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>5</v>
       </c>
-      <c r="I2">
-        <v>1</v>
-      </c>
       <c r="J2">
         <v>1</v>
       </c>
@@ -532,25 +547,87 @@
         <v>1</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="M2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="Q2">
         <v>10</v>
       </c>
-      <c r="Q2">
-        <v>0</v>
-      </c>
       <c r="R2">
-        <v>0</v>
+        <v>1.5</v>
+      </c>
+      <c r="S2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>1000102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3">
+        <v>10102</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>5</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>0.2</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>1</v>
+      </c>
+      <c r="P3">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="Q3">
+        <v>10</v>
+      </c>
+      <c r="R3">
+        <v>1.5</v>
+      </c>
+      <c r="S3">
+        <v>1.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
tối ưu monster id
</commit_message>
<xml_diff>
--- a/rollforever/Assets/Excels/MonsterConfig.xlsx
+++ b/rollforever/Assets/Excels/MonsterConfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Idle-rpg\rollforever\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD0554FE-98AA-413D-AFBC-0C08A52DFAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41B829AB-C9A7-4E4C-B609-2AF61C57B598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="9892" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>id</t>
   </si>
@@ -39,15 +39,6 @@
     <t>skill_id</t>
   </si>
   <si>
-    <t>skill_cooldown</t>
-  </si>
-  <si>
-    <t>skill_scale_damage</t>
-  </si>
-  <si>
-    <t>skill_flat_damage</t>
-  </si>
-  <si>
     <t>move_speed</t>
   </si>
   <si>
@@ -84,19 +75,19 @@
     <t>Monster 1</t>
   </si>
   <si>
-    <t>1000101_prefab</t>
-  </si>
-  <si>
     <t>Monster 2</t>
   </si>
   <si>
-    <t>1000102_prefab</t>
-  </si>
-  <si>
     <t>type</t>
   </si>
   <si>
     <t>Tanker</t>
+  </si>
+  <si>
+    <t>1001_monster</t>
+  </si>
+  <si>
+    <t>1002_monster</t>
   </si>
 </sst>
 </file>
@@ -430,35 +421,32 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="2" width="11.84375" customWidth="1"/>
     <col min="3" max="3" width="10.84375" customWidth="1"/>
     <col min="4" max="4" width="17.61328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.15234375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.23046875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.84375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.3828125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.53515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.3828125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.69140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.23046875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.4609375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.84375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="16.3828125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.61328125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.84375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.3828125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.53515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.53515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17.3828125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.69140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.23046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.4609375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.84375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.3828125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.61328125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.84375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.3828125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.53515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="16.3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:16" ht="16.3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -502,25 +490,16 @@
       <c r="P1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A2">
+        <v>1001</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
         <v>15</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A2">
-        <v>1000101</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
       </c>
       <c r="D2" t="s">
         <v>19</v>
@@ -529,104 +508,86 @@
         <v>10101</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G2">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I2">
+        <v>0.2</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="N2">
+        <v>10</v>
+      </c>
+      <c r="O2">
+        <v>1.5</v>
+      </c>
+      <c r="P2">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.4">
+      <c r="A3">
+        <v>1002</v>
+      </c>
+      <c r="B3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3">
+        <v>10201</v>
+      </c>
+      <c r="F3">
         <v>5</v>
       </c>
-      <c r="J2">
+      <c r="G3">
         <v>5</v>
       </c>
-      <c r="K2">
-        <v>1</v>
-      </c>
-      <c r="L2">
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
         <v>0.2</v>
       </c>
-      <c r="M2">
-        <v>1</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>1</v>
-      </c>
-      <c r="P2">
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
         <v>1.1000000000000001</v>
       </c>
-      <c r="Q2">
+      <c r="N3">
         <v>10</v>
       </c>
-      <c r="R2">
+      <c r="O3">
         <v>1.5</v>
       </c>
-      <c r="S2">
-        <v>1.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.4">
-      <c r="A3">
-        <v>1000102</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3">
-        <v>10102</v>
-      </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-      <c r="H3">
-        <v>1</v>
-      </c>
-      <c r="I3">
-        <v>5</v>
-      </c>
-      <c r="J3">
-        <v>5</v>
-      </c>
-      <c r="K3">
-        <v>1</v>
-      </c>
-      <c r="L3">
-        <v>0.2</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3">
-        <v>1</v>
-      </c>
-      <c r="O3">
-        <v>1</v>
-      </c>
       <c r="P3">
-        <v>1.1000000000000001</v>
-      </c>
-      <c r="Q3">
-        <v>10</v>
-      </c>
-      <c r="R3">
-        <v>1.5</v>
-      </c>
-      <c r="S3">
         <v>1.2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
save code stop distance size (v2)
</commit_message>
<xml_diff>
--- a/rollforever/Assets/Excels/MonsterConfig.xlsx
+++ b/rollforever/Assets/Excels/MonsterConfig.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Idle-rpg\rollforever\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6AC02C7-7F81-47C7-A94F-A7B1A21766E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBB1831-E71E-4E51-A1C9-625F914107A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4250" yWindow="1270" windowWidth="14400" windowHeight="8210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="baseData" sheetId="1" r:id="rId1"/>
@@ -499,7 +499,7 @@
         <v>1</v>
       </c>
       <c r="F2">
-        <v>5</v>
+        <v>0.75</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -546,7 +546,7 @@
         <v>1</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>0.75</v>
       </c>
       <c r="G3">
         <v>1</v>

</xml_diff>

<commit_message>
sửa lại phần giới hạn
</commit_message>
<xml_diff>
--- a/rollforever/Assets/Excels/MonsterConfig.xlsx
+++ b/rollforever/Assets/Excels/MonsterConfig.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Idle-rpg\rollforever\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FBB1831-E71E-4E51-A1C9-625F914107A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4034101D-9C0F-42A1-9307-CD18C7E3B006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -496,7 +496,7 @@
         <v>10101</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F2">
         <v>0.75</v>
@@ -543,7 +543,7 @@
         <v>10201</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3">
         <v>0.75</v>

</xml_diff>